<commit_message>
Create new regions in the excel-sheets
</commit_message>
<xml_diff>
--- a/data/raw/Region.xlsx
+++ b/data/raw/Region.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noemivillars-amberg/Documents/daschland-scripts/data/Spreadsheet_Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noemivillars-amberg/Documents/Customer_Projects/daschland-scripts/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{152362B2-6BF1-5C4B-A9A6-E2716286729A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA250F0D-D2BE-264F-BB7D-FCFF43B6C81F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20020" yWindow="660" windowWidth="29180" windowHeight="21880" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="47360" yWindow="600" windowWidth="29180" windowHeight="21880" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="39">
   <si>
     <t>ID</t>
   </si>
@@ -103,13 +103,52 @@
   </si>
   <si>
     <t>I_032</t>
+  </si>
+  <si>
+    <t>R_008</t>
+  </si>
+  <si>
+    <t>R_009</t>
+  </si>
+  <si>
+    <t>R_010</t>
+  </si>
+  <si>
+    <t>I_011</t>
+  </si>
+  <si>
+    <t>I_013</t>
+  </si>
+  <si>
+    <t>I_023</t>
+  </si>
+  <si>
+    <t>I_024</t>
+  </si>
+  <si>
+    <t>Cheshire Cat's tree</t>
+  </si>
+  <si>
+    <t>#3368ff</t>
+  </si>
+  <si>
+    <t>White Rabbit's house</t>
+  </si>
+  <si>
+    <t>#54ff33</t>
+  </si>
+  <si>
+    <t>R_011</t>
+  </si>
+  <si>
+    <t>R_012</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -145,6 +184,18 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -166,12 +217,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -365,13 +417,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="11.5" customWidth="1"/>
     <col min="4" max="4" width="21" customWidth="1"/>
     <col min="5" max="5" width="11.5" customWidth="1"/>
-    <col min="6" max="6" width="31" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="31.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -516,7 +568,7 @@
         <v>0.05</v>
       </c>
       <c r="D6">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="E6">
         <v>0.95</v>
@@ -583,7 +635,138 @@
         <v>23</v>
       </c>
     </row>
+    <row r="9" spans="1:8" ht="18" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9">
+        <v>0.01</v>
+      </c>
+      <c r="D9">
+        <v>0.01</v>
+      </c>
+      <c r="E9">
+        <v>0.5</v>
+      </c>
+      <c r="F9">
+        <v>0.5</v>
+      </c>
+      <c r="G9" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="18" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10">
+        <v>0.02</v>
+      </c>
+      <c r="D10">
+        <v>0.1</v>
+      </c>
+      <c r="E10">
+        <v>0.98</v>
+      </c>
+      <c r="F10">
+        <v>0.9</v>
+      </c>
+      <c r="G10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="18" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11">
+        <v>0.1</v>
+      </c>
+      <c r="D11">
+        <v>0.6</v>
+      </c>
+      <c r="E11">
+        <v>0.8</v>
+      </c>
+      <c r="F11">
+        <v>0.95</v>
+      </c>
+      <c r="G11" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="18" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12">
+        <v>0.02</v>
+      </c>
+      <c r="D12">
+        <v>0.02</v>
+      </c>
+      <c r="E12">
+        <v>0.95</v>
+      </c>
+      <c r="F12">
+        <v>0.5</v>
+      </c>
+      <c r="G12" t="s">
+        <v>33</v>
+      </c>
+      <c r="H12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="18" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13">
+        <v>0.02</v>
+      </c>
+      <c r="D13">
+        <v>0.02</v>
+      </c>
+      <c r="E13">
+        <v>0.95</v>
+      </c>
+      <c r="F13">
+        <v>0.95</v>
+      </c>
+      <c r="G13" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" t="s">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>